<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.002-06 Le sac à pain de Nino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.002-06.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.002-06.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Le sac à pain est vide. Nino veut un pain doré. D'abord un tour au jardin : oiseau, feuille froide. Le manteau gris au crochet. Le sac vide pendait sur le manteau. À la boulangerie il se souvient. Le pain rentre chaud.</t>
+          <t>Le tic de l'horloge répond dans le cuivre. Un éclat d'horloge cligne sur le sac à pain vide. Nino veut le pain du fournil, maintenant. Il court sans manteau : le sac accroche le crochet, tombe. Il refuse de forcer, enfile le gris, passe au thym. Au fournil, il pousse trop vite. Il refuse de foncer, retrouve l'éclat sur la croûte. Le sac paie le début.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un sac à pain vide pend à une chaise. Des miettes dorment sur la planche. L'horloge de la cuisine avance doucement. Une mouche marche sur la vitre. Maman s'essuie les mains dans un torchon. Nino, tu as vu le sac vide ? Oui. Il n'y a plus de pain. En ce moment, Nino souffle sur les miettes. Son manteau gris attend au crochet. L'horloge dit qu'il est tôt. On va d'abord au jardin. On verra si l'oiseau est là. Nino va vers le crochet. Le sac vide pendait aussi au crochet. Il cache un peu le manteau. Le sac est devant. Enlève le sac d'abord. Puis le manteau. Nino pose le sac sur la chaise. Il prend le manteau gris. Il est un peu épais. Nino glisse un bras, puis l'autre. Tu as pris ton manteau ? Oui, maman. Maman lace les chaussures. Ils vont au jardin. L'air est frais. Nino touche une feuille lisse. Elle est froide, maman. Oui. L'air est frais. Un oiseau picore près de la haie. Nino l'écoute un moment. Tu as vu l'oiseau ? Oui. Il picore. C'est l'heure de rentrer. Nino entre. Il retire le manteau. Il le raccroche au crochet. Le manteau gris est à sa place. Plus tard, maman prend le sac vide. On va à la boulangerie. Nino se souvient. Avant de sortir, il prend le manteau. Le même manteau gris. Tu t'es souvenu tout seul. À la boulangerie, ça sent le pain chaud. La vitrine est un peu embuée. Le pain est doré. Oui. On en prend un. Maman glisse le pain dans le sac. Puis ils rentrent. Nino raccroche encore le manteau. Le crochet fait le même petit bruit. Deux fois, maman. Oui. Deux fois. Nino pose le sac à pain sur la chaise. Le pain est encore un peu chaud. Tu as fini de poser le sac ? Oui, maman.</t>
+          <t>Le tic de l'horloge répond dans le cuivre de la casserole. La casserole est vide, froide sous le doigt. Nino connaît cette cuisine, ses recoins. Un filet de farine dessine un chemin sur la table. Sur la chaise, un sac à pain pend, vide. Le lin du sac sent la farine sèche. Un éclat d'horloge cligne sur le lin. Nino ne sait pas à quoi il servira. Maman plie le torchon, près de la planche. Le torchon sent le levain. La porte du jardin laisse un filet d'air. Ça sent le fournil du village. Nino, tu as vu le sac vide ? Oui. Il n'y a plus de pain. Je veux le pain, maintenant ! On y va, avec le sac. En ce moment, Nino saisit le sac vide. Le lin est rêche sous les doigts. Son manteau gris attend au crochet. Les pieds de Nino tapent le carrelage. Je sors, maman ! Nino court vers la porte du jardin. Il veut le pain, sans attendre. Le sac accroche le crochet, d'un coup. Oh. Nino tire plus fort. Le sac tombe, plat, sur le carrelage. Ça reste coincé ! La sangle reste tordue, près du crochet. Le manteau gris n'a pas bougé. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'air du jardin pique les poignets, sans manteau. Maman se baisse à sa hauteur. Tu regardes le crochet ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un sac à pain vide pend à une chaise. Des miettes dorment sur la planche. L'horloge de la cuisine avance doucement. Une mouche marche sur la vitre. Maman s'essuie les mains dans un torchon. Nino, tu as vu le sac vide ? Oui. Il n'y a plus de pain. En ce moment, Nino souffle sur les miettes. Son manteau gris attend au crochet. L'horloge dit qu'il est tôt. On va d'abord au jardin. On verra si l'oiseau est là. Nino va vers le crochet. Le sac vide pendait aussi au crochet. Il cache un peu le manteau. Le sac est devant. Enlève le sac d'abord. Puis le manteau. Nino pose le sac sur la chaise. Il prend le manteau gris. Il est un peu épais. Nino glisse un bras, puis l'autre. Tu as pris ton manteau ? Oui, maman. Maman lace les chaussures. Ils vont au jardin. L'air est frais. Nino touche une feuille lisse. Elle est froide, maman. Oui. L'air est frais. Un oiseau picore près de la haie. Nino l'écoute un moment. Tu as vu l'oiseau ? Oui. Il picore. C'est l'heure de rentrer. Nino entre. Il retire le manteau. Il le raccroche au crochet. Le manteau gris est à sa place. Plus tard, maman prend le sac vide. On va à la boulangerie. Nino se souvient. Avant de sortir, il prend le manteau. Le même manteau gris. Tu t'es souvenu tout seul. À la boulangerie, ça sent le pain chaud. La vitrine est un peu embuée. Le pain est doré. Oui. On en prend un. Maman glisse le pain dans le sac. Puis ils rentrent. Nino raccroche encore le manteau. Le crochet fait le même petit bruit. Deux fois, maman. Oui. Deux fois. Nino pose le sac à pain sur la chaise. Le pain est encore un peu chaud. Tu as fini de poser le sac ? Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le tic de l'horloge répond dans le cuivre de la casserole. La casserole est vide, froide sous le doigt. Nino connaît cette cuisine, ses recoins. Un filet de farine dessine un chemin sur la table. Sur la chaise, un sac à pain pend, vide. Le lin du sac sent la farine sèche. Un &lt;emphasis level="moderate"&gt;éclat d'horloge&lt;/emphasis&gt; cligne sur le lin. Nino ne sait pas à quoi il servira. Maman plie le torchon, près de la planche. Le torchon sent le levain. La porte du jardin laisse un filet d'air. Ça sent le fournil du village. Nino, tu as vu le sac vide ? Oui. Il n'y a plus de pain. Je veux le pain, maintenant ! On y va, avec le sac. En ce moment, Nino saisit le sac vide. Le lin est rêche sous les doigts. Son manteau gris attend au crochet. Les pieds de Nino tapent le carrelage. Je sors, maman ! Nino court vers la porte du jardin. Il veut le pain, sans attendre. Le sac accroche le crochet, d'un coup. Oh. Nino tire plus fort. Le sac tombe, plat, sur le carrelage. Ça reste coincé ! La sangle reste tordue, près du crochet. Le manteau gris n'a pas bougé. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'air du jardin pique les poignets, sans manteau. Maman se baisse à sa hauteur. Tu regardes le crochet ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Brice est près de la porte. Maman lace ses chaussures. Maman dit : on va au jardin. Avant de sortir, Brice prend son &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Le manteau est gris. Il est un peu épais. Brice glisse un bras, puis l'autre. Ils vont au jardin. L'air est frais. Brice touche une feuille lisse. Maman dit : on rentre. Brice entre. Il retire le manteau. Il le raccroche au crochet. Le manteau est à sa place. Plus tard, maman dit : on va à la boulangerie. Brice se souvient. Avant de sortir, il prend le manteau. À la boulangerie, ça sent le pain. Puis ils rentrent. Brice raccroche encore le manteau. Même leçon, autre sortie. Maman dit : merci Brice. [pause]</t>
+          <t>Le tic de l'horloge répond dans le cuivre de la casserole. La casserole est vide, froide sous le doigt. Nino connaît cette cuisine, ses recoins. Un filet de farine dessine un chemin sur la table. Sur la chaise, un sac à pain pend, vide. Le lin du sac sent la farine sèche. Un &lt;emphasis&gt;éclat d'horloge&lt;/emphasis&gt; cligne sur le lin. Nino ne sait pas à quoi il servira. Maman plie le torchon, près de la planche. Le torchon sent le levain. La porte du jardin laisse un filet d'air. Ça sent le fournil du village. Nino, tu as vu le sac vide ? Oui. Il n'y a plus de pain. Je veux le pain, maintenant ! On y va, avec le sac. En ce moment, Nino saisit le sac vide. Le lin est rêche sous les doigts. Son manteau gris attend au crochet. Les pieds de Nino tapent le carrelage. Je sors, maman ! Nino court vers la porte du jardin. Il veut le pain, sans attendre. Le sac accroche le crochet, d'un coup. Oh. Nino tire plus fort. Le sac tombe, plat, sur le carrelage. Ça reste coincé ! La sangle reste tordue, près du crochet. Le manteau gris n'a pas bougé. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. L'air du jardin pique les poignets, sans manteau. Maman se baisse à sa hauteur. Tu regardes le crochet ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>éclat d'horloge</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,78 +1321,54 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_pain_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un sac à pain vide pend à une chaise.
-narrateur|Des miettes dorment sur la planche.
-narrateur|L'horloge de la cuisine avance doucement.
-narrateur|Une mouche marche sur la vitre.
-narrateur|Maman s'essuie les mains dans un torchon.
+          <t>narrateur|Le tic de l'horloge répond dans le cuivre de la casserole.
+narrateur|La casserole est vide, froide sous le doigt.
+narrateur|Nino connaît cette cuisine, ses recoins.
+narrateur|Un filet de farine dessine un chemin sur la table.
+narrateur|Sur la chaise, un sac à pain pend, vide.
+narrateur|Le lin du sac sent la farine sèche.
+narrateur|Un éclat d'horloge cligne sur le lin.
+narrateur|Nino ne sait pas à quoi il servira.
+narrateur|Maman plie le torchon, près de la planche.
+narrateur|Le torchon sent le levain.
+narrateur|La porte du jardin laisse un filet d'air.
+narrateur|Ça sent le fournil du village.
 maman|Nino, tu as vu le sac vide ?
 enfant-m|Oui.
 enfant-m|Il n'y a plus de pain.
-narrateur|En ce moment, Nino souffle sur les miettes.
+enfant-m|Je veux le pain, maintenant !
+maman|On y va, avec le sac.
+narrateur|En ce moment, Nino saisit le sac vide.
+narrateur|Le lin est rêche sous les doigts.
 narrateur|Son manteau gris attend au crochet.
-maman|L'horloge dit qu'il est tôt.
-maman|On va d'abord au jardin.
-maman|On verra si l'oiseau est là.
-narrateur|Nino va vers le crochet.
-narrateur|Le sac vide pendait aussi au crochet.
-narrateur|Il cache un peu le manteau.
-enfant-m|Le sac est devant.
-maman|Enlève le sac d'abord.
-maman|Puis le manteau.
-narrateur|Nino pose le sac sur la chaise.
-narrateur|Il prend le manteau gris.
-narrateur|Il est un peu épais.
-narrateur|Nino glisse un bras, puis l'autre.
-maman|Tu as pris ton manteau ?
-enfant-m|Oui, maman.
-narrateur|Maman lace les chaussures.
-narrateur|Ils vont au jardin.
-narrateur|L'air est frais.
-narrateur|Nino touche une feuille lisse.
-enfant-m|Elle est froide, maman.
-maman|Oui.
-maman|L'air est frais.
-narrateur|Un oiseau picore près de la haie.
-narrateur|Nino l'écoute un moment.
-maman|Tu as vu l'oiseau ?
-enfant-m|Oui.
-enfant-m|Il picore.
-maman|C'est l'heure de rentrer.
-narrateur|Nino entre.
-narrateur|Il retire le manteau.
-narrateur|Il le raccroche au crochet.
-narrateur|Le manteau gris est à sa place.
-narrateur|Plus tard, maman prend le sac vide.
-maman|On va à la boulangerie.
-narrateur|Nino se souvient.
-narrateur|Avant de sortir, il prend le manteau.
-narrateur|Le même manteau gris.
-maman|Tu t'es souvenu tout seul.
-narrateur|À la boulangerie, ça sent le pain chaud.
-narrateur|La vitrine est un peu embuée.
-enfant-m|Le pain est doré.
-maman|Oui.
-maman|On en prend un.
-narrateur|Maman glisse le pain dans le sac.
-narrateur|Puis ils rentrent.
-narrateur|Nino raccroche encore le manteau.
-narrateur|Le crochet fait le même petit bruit.
-enfant-m|Deux fois, maman.
-maman|Oui.
-maman|Deux fois.
-narrateur|Nino pose le sac à pain sur la chaise.
-narrateur|Le pain est encore un peu chaud.
-maman|Tu as fini de poser le sac ?
-enfant-m|Oui, maman.</t>
+narrateur|Les pieds de Nino tapent le carrelage.
+enfant-m|Je sors, maman !
+narrateur|Nino court vers la porte du jardin.
+narrateur|Il veut le pain, sans attendre.
+narrateur|Le sac accroche le crochet, d'un coup.
+enfant-m|Oh.
+narrateur|Nino tire plus fort.
+narrateur|Le sac tombe, plat, sur le carrelage.
+enfant-m|Ça reste coincé !
+narrateur|La sangle reste tordue, près du crochet.
+narrateur|Le manteau gris n'a pas bougé.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|L'air du jardin pique les poignets, sans manteau.
+narrateur|Maman se baisse à sa hauteur.
+maman|Tu regardes le crochet ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>horloge,porte</t>
+          <t>horloge,casserole,porte</t>
         </is>
       </c>
     </row>
@@ -1419,17 +1395,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Nino ?</t>
+          <t>Nino veut sortir. Avant de sortir, que prend Nino ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Nino ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino veut &lt;emphasis level="moderate"&gt;sortir&lt;/emphasis&gt;. Avant de sortir, que prend Nino ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Avant de &lt;emphasis&gt;sortir&lt;/emphasis&gt;, que prend Brice ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino veut &lt;emphasis&gt;sortir&lt;/emphasis&gt;. Avant de sortir, que prend Nino ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1492,7 +1468,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1500,10 +1476,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1518,11 +1494,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1533,23 +1509,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1558,28 +1534,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_manteau_avant_la_porte; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de sortir, que prend Nino ?</t>
+          <t>narrateur|Nino veut sortir.
+narrateur|Avant de sortir, que prend Nino ?</t>
         </is>
       </c>
     </row>
@@ -1606,17 +1583,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino a pris le manteau. Au jardin, puis à la boulangerie. Deux sorties. Le même manteau gris. En rentrant, il l'a raccroché. Tu t'es souvenu. Il est au crochet. Oui.</t>
+          <t>Nino refuse de tirer plus fort. Il pose un genou au carrelage. Le sac est plat, la sangle tordue. Je le pose. Il pose le sac sur la chaise. Le crochet montre le manteau gris. Tu le prends, Nino ? Oui, maman. Nino glisse un bras, puis l'autre. Le tissu est épais, un peu rêche. Les boutons sont froids sous le doigt. Merci, Nino. Le manteau est prêt ? Oui, maman. Maman lace les chaussures, sans se presser. On ouvre le jardin ? Oui. Ils passent la porte du jardin. L'air pique les joues, pas les poignets. J'ai chaud, maman. Tu le sens sur tes bras ? Oui. Un arrosoir goutte près du thym. Le thym sent fort, près de la grille. Il goutte, maman. Tu l'entends, Nino ? Nino écoute la goutte, un instant. La grille du jardin grince, un peu. On rentre. Nino entre. Il retire le manteau gris. Il le raccroche au crochet. Il est à sa place.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nino a pris le manteau. Au jardin, puis à la boulangerie. Deux sorties. Le même manteau gris. En rentrant, il l'a raccroché. Tu t'es souvenu. Il est au crochet. Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino refuse de tirer plus fort. Il pose un genou au carrelage. Le sac est plat, la sangle tordue. Je le pose. Il pose le sac sur la chaise. Le crochet montre le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt; gris. Tu le prends, Nino ? Oui, maman. Nino glisse un bras, puis l'autre. Le tissu est épais, un peu rêche. Les boutons sont froids sous le doigt. Merci, Nino. Le manteau est prêt ? Oui, maman. Maman lace les chaussures, sans se presser. On ouvre le jardin ? Oui. Ils passent la porte du jardin. L'air pique les joues, pas les poignets. J'ai chaud, maman. Tu le sens sur tes bras ? Oui. Un arrosoir goutte près du thym. Le thym sent fort, près de la grille. Il goutte, maman. Tu l'entends, Nino ? Nino écoute la goutte, un instant. La grille du jardin grince, un peu. On rentre. Nino entre. Il retire le manteau gris. Il le raccroche au crochet. Il est à sa place.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Brice a pris le &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Au jardin, puis à la boulangerie. En rentrant, il l'a raccroché. [pause]</t>
+          <t>Nino refuse de tirer plus fort. Il pose un genou au carrelage. Le sac est plat, la sangle tordue. Je le pose. Il pose le sac sur la chaise. Le crochet montre le &lt;emphasis&gt;manteau&lt;/emphasis&gt; gris. Tu le prends, Nino ? Oui, maman. Nino glisse un bras, puis l'autre. Le tissu est épais, un peu rêche. Les boutons sont froids sous le doigt. Merci, Nino. Le manteau est prêt ? Oui, maman. Maman lace les chaussures, sans se presser. On ouvre le jardin ? Oui. Ils passent la porte du jardin. L'air pique les joues, pas les poignets. J'ai chaud, maman. Tu le sens sur tes bras ? Oui. Un arrosoir goutte près du thym. Le thym sent fort, près de la grille. Il goutte, maman. Tu l'entends, Nino ? Nino écoute la goutte, un instant. La grille du jardin grince, un peu. On rentre. Nino entre. Il retire le manteau gris. Il le raccroche au crochet. Il est à sa place. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1663,7 +1640,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1671,10 +1648,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1704,23 +1681,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1729,10 +1706,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1745,19 +1722,49 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_prend_le_manteau_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino a pris le manteau.
-narrateur|Au jardin, puis à la boulangerie.
-narrateur|Deux sorties.
-narrateur|Le même manteau gris.
-narrateur|En rentrant, il l'a raccroché.
-maman|Tu t'es souvenu.
-enfant-m|Il est au crochet.
-maman|Oui.</t>
+          <t>narrateur|Nino refuse de tirer plus fort.
+narrateur|Il pose un genou au carrelage.
+narrateur|Le sac est plat, la sangle tordue.
+enfant-m|Je le pose.
+narrateur|Il pose le sac sur la chaise.
+narrateur|Le crochet montre le manteau gris.
+maman|Tu le prends, Nino ?
+enfant-m|Oui, maman.
+narrateur|Nino glisse un bras, puis l'autre.
+narrateur|Le tissu est épais, un peu rêche.
+narrateur|Les boutons sont froids sous le doigt.
+maman|Merci, Nino.
+maman|Le manteau est prêt ?
+enfant-m|Oui, maman.
+narrateur|Maman lace les chaussures, sans se presser.
+maman|On ouvre le jardin ?
+enfant-m|Oui.
+narrateur|Ils passent la porte du jardin.
+narrateur|L'air pique les joues, pas les poignets.
+enfant-m|J'ai chaud, maman.
+maman|Tu le sens sur tes bras ?
+enfant-m|Oui.
+narrateur|Un arrosoir goutte près du thym.
+narrateur|Le thym sent fort, près de la grille.
+enfant-m|Il goutte, maman.
+maman|Tu l'entends, Nino ?
+narrateur|Nino écoute la goutte, un instant.
+narrateur|La grille du jardin grince, un peu.
+maman|On rentre.
+narrateur|Nino entre.
+narrateur|Il retire le manteau gris.
+narrateur|Il le raccroche au crochet.
+enfant-m|Il est à sa place.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>manteau,jardin,arrosoir</t>
         </is>
       </c>
     </row>
@@ -1784,17 +1791,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino pose les chaussures. Le manteau reste au crochet. Maman pose le pain sur la planche. Tu as fini de poser tes chaussures ? Oui, maman. Le sac n'est plus vide. Les miettes nouvelles sentent le chaud. On a le pain, maintenant. Et le manteau est à sa place. Oui.</t>
+          <t>On prend le sac, Nino ? Le pain, maintenant. Maman prend le sac vide. Nino va vers le crochet, seul. Il prend le manteau gris. Le manteau, maman. Tu l'as pris, toi. Ils traversent le jardin, puis la rue. Le fournil sent le chaud, si près. Je le prends ! Nino pousse la porte, trop vite. Le sac se coince dans le battant. Oh. Il veut foncer vers le pain chaud. Nino refuse de foncer. Attends, je regarde. Au-dessus du comptoir, un cadran brille. Un éclat d'horloge cligne sur la croûte. Comme à la cuisine ! Tu le vois, toi ? Oui, sur ce pain. Nino s'arrête, lent. Il écoute le fournil, un instant. Une pelle racle la pierre, plus loin. Le pain attend derrière le bois. On le prend ensemble ? Celui-là.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino pose les chaussures. Le manteau reste au crochet. Maman pose le pain sur la planche. Tu as fini de poser tes chaussures ? Oui, maman. Le sac n'est plus vide. Les miettes nouvelles sentent le chaud. On a le pain, maintenant. Et le manteau est à sa place. Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;On prend le sac, Nino ? Le pain, maintenant. Maman prend le sac vide. Nino va vers le crochet, seul. Il prend le manteau gris. Le manteau, maman. Tu l'as pris, toi. Ils traversent le jardin, puis la rue. Le fournil sent le chaud, si près. Je le prends ! Nino pousse la porte, trop vite. Le sac se coince dans le battant. Oh. Il veut foncer vers le pain chaud. Nino refuse de foncer. Attends, je regarde. Au-dessus du comptoir, un cadran brille. Un &lt;emphasis level="moderate"&gt;éclat d'horloge&lt;/emphasis&gt; cligne sur la croûte. Comme à la cuisine ! Tu le vois, toi ? Oui, sur ce pain. Nino s'arrête, lent. Il écoute le fournil, un instant. Une pelle racle la pierre, plus loin. Le pain attend derrière le bois. On le prend ensemble ? Celui-là.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Brice pose les chaussures. Le &lt;emphasis&gt;manteau&lt;/emphasis&gt; reste au crochet. [pause]</t>
+          <t>&lt;low-pitch&gt;On prend le sac, Nino ? Le pain, maintenant. Maman prend le sac vide. Nino va vers le crochet, seul. Il prend le manteau gris. Le manteau, maman. Tu l'as pris, toi. Ils traversent le jardin, puis la rue. Le fournil sent le chaud, si près. Je le prends ! Nino pousse la porte, trop vite. Le sac se coince dans le battant. Oh. Il veut foncer vers le pain chaud. Nino refuse de foncer. Attends, je regarde. Au-dessus du comptoir, un cadran brille. Un &lt;emphasis&gt;éclat d'horloge&lt;/emphasis&gt; cligne sur la croûte. Comme à la cuisine ! Tu le vois, toi ? Oui, sur ce pain. Nino s'arrête, lent. Il écoute le fournil, un instant. Une pelle racle la pierre, plus loin. Le pain attend derrière le bois. On le prend ensemble ? Celui-là.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1841,7 +1848,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1849,22 +1856,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1875,30 +1886,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>éclat d'horloge</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1907,33 +1918,59 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nino pose les chaussures.
-narrateur|Le manteau reste au crochet.
-narrateur|Maman pose le pain sur la planche.
-maman|Tu as fini de poser tes chaussures ?
-enfant-m|Oui, maman.
-narrateur|Le sac n'est plus vide.
-narrateur|Les miettes nouvelles sentent le chaud.
-maman|On a le pain, maintenant.
-enfant-m|Et le manteau est à sa place.
-maman|Oui.</t>
+          <t>maman|On prend le sac, Nino ?
+enfant-m|Le pain, maintenant.
+narrateur|Maman prend le sac vide.
+narrateur|Nino va vers le crochet, seul.
+narrateur|Il prend le manteau gris.
+enfant-m|Le manteau, maman.
+maman|Tu l'as pris, toi.
+narrateur|Ils traversent le jardin, puis la rue.
+narrateur|Le fournil sent le chaud, si près.
+enfant-m|Je le prends !
+narrateur|Nino pousse la porte, trop vite.
+narrateur|Le sac se coince dans le battant.
+enfant-m|Oh.
+narrateur|Il veut foncer vers le pain chaud.
+narrateur|Nino refuse de foncer.
+enfant-m|Attends, je regarde.
+narrateur|Au-dessus du comptoir, un cadran brille.
+narrateur|Un éclat d'horloge cligne sur la croûte.
+enfant-m|Comme à la cuisine !
+maman|Tu le vois, toi ?
+enfant-m|Oui, sur ce pain.
+narrateur|Nino s'arrête, lent.
+narrateur|Il écoute le fournil, un instant.
+narrateur|Une pelle racle la pierre, plus loin.
+narrateur|Le pain attend derrière le bois.
+maman|On le prend ensemble ?
+enfant-m|Celui-là.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>porte,fournil,pelle</t>
         </is>
       </c>
     </row>
@@ -1960,17 +1997,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai pris le manteau deux fois. Jardin, puis boulangerie. Et tu l'as raccroché. Bravo, Nino. Le pain doré attend sur la planche.</t>
+          <t>Maman glisse le pain dans le sac. Le lin se tend, un peu chaud. Il sent le fournil, maman. Tu le portes, toi ? Oui, contre moi. Nino serre le sac contre le manteau. Sur la croûte, l'éclat d'horloge reste. Comme sur le lin, maman. Tu le ramènes à la maison ? Oui. Ils rentrent par le jardin. Nino raccroche le manteau au crochet. Le sac repose sur la chaise. Il n'est plus vide. Tu as fini de poser le sac ? Oui, maman. L'éclat d'horloge laisse une trace claire, sur la croûte.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai pris le manteau deux fois. Jardin, puis boulangerie. Et tu l'as raccroché. Bravo, Nino. Le pain doré attend sur la planche.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Maman glisse le pain dans le sac. Le lin se tend, un peu chaud. Il sent le fournil, maman. Tu le portes, toi ? Oui, contre moi. Nino serre le sac contre le manteau. Sur la croûte, l'&lt;emphasis level="moderate"&gt;éclat d'horloge&lt;/emphasis&gt; reste. Comme sur le lin, maman. Tu le ramènes à la maison ? Oui. Ils rentrent par le jardin. Nino raccroche le manteau au crochet. Le sac repose sur la chaise. Il n'est plus vide. Tu as fini de poser le sac ? Oui, maman. L'éclat d'horloge laisse une trace claire, sur la croûte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Maman glisse le pain dans le sac. Le lin se tend, un peu chaud. Il sent le fournil, maman. Tu le portes, toi ? Oui, contre moi. Nino serre le sac contre le manteau. Sur la croûte, l'&lt;emphasis&gt;éclat d'horloge&lt;/emphasis&gt; reste. Comme sur le lin, maman. Tu le ramènes à la maison ? Oui. Ils rentrent par le jardin. Nino raccroche le manteau au crochet. Le sac repose sur la chaise. Il n'est plus vide. Tu as fini de poser le sac ? Oui, maman. L'éclat d'horloge laisse une trace claire, sur la croûte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2017,15 +2054,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2037,12 +2074,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2051,17 +2088,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'horloge</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2070,11 +2111,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2083,28 +2124,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_cadran_est_sur_la_croute; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai pris le manteau deux fois.
-enfant-m|Jardin, puis boulangerie.
-maman|Et tu l'as raccroché.
-maman|Bravo, Nino.
-narrateur|Le pain doré attend sur la planche.</t>
+          <t>narrateur|Maman glisse le pain dans le sac.
+narrateur|Le lin se tend, un peu chaud.
+enfant-m|Il sent le fournil, maman.
+maman|Tu le portes, toi ?
+enfant-m|Oui, contre moi.
+narrateur|Nino serre le sac contre le manteau.
+narrateur|Sur la croûte, l'éclat d'horloge reste.
+enfant-m|Comme sur le lin, maman.
+maman|Tu le ramènes à la maison ?
+enfant-m|Oui.
+narrateur|Ils rentrent par le jardin.
+narrateur|Nino raccroche le manteau au crochet.
+narrateur|Le sac repose sur la chaise.
+enfant-m|Il n'est plus vide.
+maman|Tu as fini de poser le sac ?
+enfant-m|Oui, maman.
+narrateur|L'éclat d'horloge laisse une trace claire, sur la croûte.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>sac,crochet</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2217,6 +2279,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>